<commit_message>
Complete Week 4 validation results
</commit_message>
<xml_diff>
--- a/outputs/week4_validation_results.xlsx
+++ b/outputs/week4_validation_results.xlsx
@@ -1215,15 +1215,15 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>A minimalist geometric illustration of a landscape featuring dark triangular mountains, a yellow sun, a pink sky, and a bl...</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1233,14 +1233,10 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1250,32 +1246,28 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>A light blue water bottle icon with a dark blue cap and the text 'H2O' on the front.</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1285,15 +1277,15 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>A simple black line icon of a key on a light gray background.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1303,14 +1295,10 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1320,30 +1308,30 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Bar chart titled Club Signups by Month showing student numbers for Jan, Feb, Mar, and Apr.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
+          <t>Hard case passed, but verify manually because the subject/text is intentionally difficult.</t>
         </is>
       </c>
     </row>
@@ -1355,30 +1343,30 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>A very dark, low-resolution image showing a faint, blurry silhouette of a person's head and shoulders against a black back...</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
+          <t>Did not capture all critical visible text or event details.</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1399,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
@@ -1426,7 +1414,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
@@ -1517,32 +1505,28 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>UW Club Fair flyer showing students visiting club tables on a sunny campus lawn.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1552,32 +1536,28 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Illustration of two students presenting a wheeled robot near a classroom table during a Robotics Demo.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1587,32 +1567,28 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Illustration of a campus food drive with four volunteers collecting donations at a table.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1622,32 +1598,28 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Announcement card for a Blood Drive on Oct 12 at the Student Union from 10 AM to 3 PM.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1657,32 +1629,28 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Event card for Coding Night on Friday at 7 PM in Room 204, with a reminder to bring a laptop.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0</v>
+        <v>93</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1692,32 +1660,28 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Event flyer for Spring Art Show on May 3 at Gallery Hall, 6 PM, with a blue circle graphic.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1727,30 +1691,30 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Illustration of a forest with a single tree stump among standing trees, symbolizing deforestation.</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
+          <t>Invented a deforestation/stump meaning that was not actually present in the image.</t>
         </is>
       </c>
     </row>
@@ -1762,15 +1726,15 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Flat vector illustration of a minimalist landscape with mountains, a yellow sun, and a pink sky over blue water.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1780,14 +1744,10 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1797,32 +1757,28 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>A light blue water bottle icon with a dark blue cap and the text 'H2O' on the front.</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1832,15 +1788,15 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>A simple black icon of a key on a light gray background, symbolizing access or security.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1850,14 +1806,10 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1867,30 +1819,30 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Bar chart showing rising club signups: 110 in Jan, 190 in Feb, 300 in Mar, 430 in Apr.</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
+          <t>Hard case passed, but verify manually because the subject/text is intentionally difficult.</t>
         </is>
       </c>
     </row>
@@ -1902,30 +1854,30 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PENDING - Groq daily token limit reached before this image could be tested.</t>
+          <t>Placeholder icon indicating a dim room with an unclear subject, used when image content is too dark to identify.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Not measured yet because Groq returned a daily token-limit error during validation.</t>
+          <t>Hard case passed, but verify manually because the subject/text is intentionally difficult.</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1910,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
@@ -1973,7 +1925,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
@@ -1988,7 +1940,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>

</xml_diff>